<commit_message>
updated the min trading value
</commit_message>
<xml_diff>
--- a/src/allocations.xlsx
+++ b/src/allocations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/brand/Desktop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1F36869-1AE6-434C-8C0A-C1DEFE4850BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{365477B3-22B5-DD4C-AA96-5B442A4D7CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="15620" xr2:uid="{BBF777D5-466C-F647-BCE9-E7DBB05CFFE3}"/>
+    <workbookView xWindow="760" yWindow="760" windowWidth="28040" windowHeight="15580" xr2:uid="{BBF777D5-466C-F647-BCE9-E7DBB05CFFE3}"/>
   </bookViews>
   <sheets>
     <sheet name="allocations" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>contract_code</t>
   </si>
@@ -52,18 +52,6 @@
     <t>"New Wave Silver ETN"</t>
   </si>
   <si>
-    <t>NGPLT</t>
-  </si>
-  <si>
-    <t>"NewPlat ETF"</t>
-  </si>
-  <si>
-    <t>STX40</t>
-  </si>
-  <si>
-    <t>"Satrix 40 ETF"</t>
-  </si>
-  <si>
     <t>EQU.ZA.STX500</t>
   </si>
   <si>
@@ -73,10 +61,13 @@
     <t>EQU.ZA.NEWSLV</t>
   </si>
   <si>
-    <t>EQU.ZA.NGPLT</t>
-  </si>
-  <si>
-    <t>EQU.ZA.STX40</t>
+    <t>EQU.ZA.EASYBF</t>
+  </si>
+  <si>
+    <t>EASYBF</t>
+  </si>
+  <si>
+    <t>"EasyETFs Balanced Actively Managed ETF"</t>
   </si>
 </sst>
 </file>
@@ -938,12 +929,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C4336C7C-0882-B649-B22A-5BEA4F945B84}">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.1640625" customWidth="1"/>
     <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="29.5" customWidth="1"/>
+    <col min="4" max="4" width="42.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
@@ -962,13 +953,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -976,13 +967,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
@@ -990,13 +981,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
       </c>
       <c r="C4">
-        <v>0.2</v>
+        <v>0.05</v>
       </c>
       <c r="D4" t="s">
         <v>9</v>
@@ -1004,30 +995,16 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C5">
-        <v>0.2</v>
+        <v>0.45</v>
       </c>
       <c r="D5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C6">
-        <v>0.2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>